<commit_message>
Add 36 conductors cable ref. RS
</commit_message>
<xml_diff>
--- a/Interface_IAI.xlsx
+++ b/Interface_IAI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Buloup\Documents\GIT\Interface_IAI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A738DB8-9050-474F-BB1D-D3B5A4C78D7F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C3A9CC6-EFAE-4699-94DD-C08D7B83BA37}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="116">
   <si>
     <t>Composants pour cicuit imprimé</t>
   </si>
@@ -352,49 +352,7 @@
     <t xml:space="preserve"> 175-3723</t>
   </si>
   <si>
-    <t>Filtre EMI (RS )</t>
-  </si>
-  <si>
     <t>292-818</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Filtre </t>
-    </r>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>EMI</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t xml:space="preserve"> (</t>
-    </r>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>RS</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t xml:space="preserve"> )</t>
-    </r>
   </si>
   <si>
     <t>708-4272</t>
@@ -521,6 +479,37 @@
   </si>
   <si>
     <t>Connecteur CEI Droit C19 Schurter, Câble</t>
+  </si>
+  <si>
+    <t>236-9258</t>
+  </si>
+  <si>
+    <t>Câble industriels multiconducteur (36 - 25m)</t>
+  </si>
+  <si>
+    <t>Filtre EMI 20A</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Filtre </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>EMI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t xml:space="preserve"> 10A</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -1497,7 +1486,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H62"/>
+  <dimension ref="A1:H63"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="45.109375" customWidth="1"/>
@@ -1533,13 +1522,13 @@
         <v>1</v>
       </c>
       <c r="B3" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="D3" s="6" t="s">
         <v>98</v>
-      </c>
-      <c r="C3" s="12" t="s">
-        <v>99</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>100</v>
       </c>
       <c r="E3" s="6" t="s">
         <v>2</v>
@@ -2275,7 +2264,7 @@
     </row>
     <row r="30" spans="1:8">
       <c r="A30" s="1" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B30" s="1">
         <v>1</v>
@@ -2335,13 +2324,13 @@
         <v>1</v>
       </c>
       <c r="B35" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C35" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="D35" s="6" t="s">
         <v>98</v>
-      </c>
-      <c r="C35" s="12" t="s">
-        <v>99</v>
-      </c>
-      <c r="D35" s="6" t="s">
-        <v>100</v>
       </c>
       <c r="E35" s="6" t="s">
         <v>2</v>
@@ -2390,7 +2379,7 @@
     </row>
     <row r="39" spans="1:8">
       <c r="A39" s="15" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B39" s="15"/>
       <c r="C39" s="15"/>
@@ -2415,13 +2404,13 @@
         <v>1</v>
       </c>
       <c r="B41" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C41" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="D41" s="6" t="s">
         <v>98</v>
-      </c>
-      <c r="C41" s="12" t="s">
-        <v>99</v>
-      </c>
-      <c r="D41" s="6" t="s">
-        <v>100</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>2</v>
@@ -2470,7 +2459,7 @@
         <v>1</v>
       </c>
       <c r="C43" s="13">
-        <f t="shared" ref="C43:C57" si="2">B43*2</f>
+        <f t="shared" ref="C43:C58" si="2">B43*2</f>
         <v>2</v>
       </c>
       <c r="D43" s="1"/>
@@ -2484,13 +2473,13 @@
         <v>7.53</v>
       </c>
       <c r="H43" s="1">
-        <f t="shared" ref="H43:H57" si="3">G43*C43</f>
+        <f t="shared" ref="H43:H58" si="3">G43*C43</f>
         <v>15.06</v>
       </c>
     </row>
     <row r="44" spans="1:8">
       <c r="A44" s="7" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B44" s="1">
         <v>0.5</v>
@@ -2516,7 +2505,7 @@
     </row>
     <row r="45" spans="1:8">
       <c r="A45" s="7" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B45" s="1">
         <v>1</v>
@@ -2530,7 +2519,7 @@
         <v>77</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="G45" s="1">
         <v>7.91</v>
@@ -2556,7 +2545,7 @@
         <v>77</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="G46" s="1">
         <v>244.52</v>
@@ -2594,7 +2583,7 @@
     </row>
     <row r="48" spans="1:8">
       <c r="A48" s="7" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B48" s="1">
         <v>0.5</v>
@@ -2620,7 +2609,7 @@
     </row>
     <row r="49" spans="1:8">
       <c r="A49" s="7" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B49" s="1">
         <v>0.5</v>
@@ -2646,7 +2635,7 @@
     </row>
     <row r="50" spans="1:8">
       <c r="A50" s="7" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B50" s="1">
         <v>0.5</v>
@@ -2672,7 +2661,7 @@
     </row>
     <row r="51" spans="1:8">
       <c r="A51" s="7" t="s">
-        <v>88</v>
+        <v>114</v>
       </c>
       <c r="B51" s="1">
         <v>0.5</v>
@@ -2686,7 +2675,7 @@
         <v>77</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G51" s="1">
         <v>67.75</v>
@@ -2698,7 +2687,7 @@
     </row>
     <row r="52" spans="1:8">
       <c r="A52" s="7" t="s">
-        <v>90</v>
+        <v>115</v>
       </c>
       <c r="B52" s="1">
         <v>0.5</v>
@@ -2712,7 +2701,7 @@
         <v>77</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="G52" s="1">
         <v>52.9</v>
@@ -2724,7 +2713,7 @@
     </row>
     <row r="53" spans="1:8">
       <c r="A53" s="7" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B53" s="1">
         <v>4</v>
@@ -2738,7 +2727,7 @@
         <v>77</v>
       </c>
       <c r="F53" s="7" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="G53" s="1">
         <v>10.46</v>
@@ -2750,7 +2739,7 @@
     </row>
     <row r="54" spans="1:8">
       <c r="A54" s="9" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B54" s="10">
         <v>1</v>
@@ -2764,7 +2753,7 @@
         <v>77</v>
       </c>
       <c r="F54" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="G54" s="10">
         <v>7.89</v>
@@ -2776,7 +2765,7 @@
     </row>
     <row r="55" spans="1:8">
       <c r="A55" s="1" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B55" s="10">
         <v>1</v>
@@ -2790,7 +2779,7 @@
         <v>77</v>
       </c>
       <c r="F55" s="10" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="G55" s="10">
         <v>4.92</v>
@@ -2802,7 +2791,7 @@
     </row>
     <row r="56" spans="1:8">
       <c r="A56" s="1" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B56" s="10">
         <v>0.5</v>
@@ -2816,7 +2805,7 @@
         <v>77</v>
       </c>
       <c r="F56" s="10" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="G56" s="10">
         <v>21.89</v>
@@ -2828,7 +2817,7 @@
     </row>
     <row r="57" spans="1:8">
       <c r="A57" s="1" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B57" s="10">
         <v>0.5</v>
@@ -2842,7 +2831,7 @@
         <v>77</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="G57" s="10">
         <v>9.83</v>
@@ -2853,35 +2842,61 @@
       </c>
     </row>
     <row r="58" spans="1:8">
-      <c r="A58" s="8"/>
+      <c r="A58" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B58" s="10">
+        <v>0.5</v>
+      </c>
+      <c r="C58" s="11">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="D58" s="11"/>
+      <c r="E58" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="F58" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="G58" s="10">
+        <v>181.19</v>
+      </c>
+      <c r="H58" s="10">
+        <f t="shared" si="3"/>
+        <v>181.19</v>
+      </c>
     </row>
     <row r="59" spans="1:8">
-      <c r="G59" s="5" t="s">
+      <c r="A59" s="8"/>
+    </row>
+    <row r="60" spans="1:8">
+      <c r="G60" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H59" s="5">
-        <f>SUM(H42:H57)</f>
-        <v>634.20999999999992</v>
-      </c>
-    </row>
-    <row r="61" spans="1:8">
-      <c r="F61" s="16" t="s">
+      <c r="H60" s="5">
+        <f>SUM(H42:H58)</f>
+        <v>815.39999999999986</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8">
+      <c r="F62" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="G61" s="17"/>
-      <c r="H61" s="3">
-        <f>H32+H38+H59</f>
-        <v>908.27</v>
-      </c>
-    </row>
-    <row r="62" spans="1:8">
-      <c r="F62" s="18" t="s">
+      <c r="G62" s="17"/>
+      <c r="H62" s="3">
+        <f>H32+H38+H60</f>
+        <v>1089.46</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8">
+      <c r="F63" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="G62" s="19"/>
-      <c r="H62" s="4">
-        <f>H61*1.2</f>
-        <v>1089.924</v>
+      <c r="G63" s="19"/>
+      <c r="H63" s="4">
+        <f>H62*1.2</f>
+        <v>1307.3520000000001</v>
       </c>
     </row>
   </sheetData>
@@ -2889,8 +2904,8 @@
     <mergeCell ref="A1:H2"/>
     <mergeCell ref="A33:H34"/>
     <mergeCell ref="A39:H40"/>
-    <mergeCell ref="F61:G61"/>
     <mergeCell ref="F62:G62"/>
+    <mergeCell ref="F63:G63"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>